<commit_message>
Week 4 open: local pipeline resync onto the merged TEN data-kit fix
Local gitignored state predated PR #1 (TEN June-5 data-kit reconcile),
so the pipeline + reconcile were re-run on the merged inputs: TEN
confirms at NAV $88.13 / gap -19.3% (the PR's numbers), 244 tests pass,
17/17 SANITY OK, single drift alert is the TEN fix itself (annotated).
STNG and SBLK band-edge position flips on the Jun-11 live closes
annotated as market wiggle, no action.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16.89</v>
+        <v>16.38</v>
       </c>
     </row>
     <row r="5">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>49486.13291402483</v>
+        <v>43209.28591109523</v>
       </c>
     </row>
     <row r="16">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.999439713697973</v>
+        <v>1.745829733781626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: pipeline-run artifacts from the BRUT onboarding + §9.6 rollout
Regenerated per-name outputs (fv reports / scenarios / broker sweep / summaries /
delta report) + routine decision-log model-state stubs from the 2026-06-22
pipeline runs (BRUT onboarding + the §9.6 time-to-delivery discount rollout to
CAPT/FRO/MPCC). Downstream of the source/input changes already committed; kept
to leave a clean tree. Outside scripts/commit_drift.sh scope by design.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16.38</v>
+        <v>17.07</v>
       </c>
     </row>
     <row r="5">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>43209.28591109523</v>
+        <v>51701.4906797647</v>
       </c>
     </row>
     <row r="16">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.745829733781626</v>
+        <v>2.088949118374331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
baseline: re-ratify drift gate — July-1 price-vintage recovery (audit F-1 follow-up; ΔNAV 0.0% all names, pure price drift; STNG flip annotated)
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -425,7 +425,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16</v>
+        <v>14.25</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18010.34170400495</v>
+        <v>1481.079857180723</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.7276905738991897</v>
+        <v>0.05984161039114032</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
baseline: re-ratify drift gate — July-2 close price drift (isolated layer)
Post-stand-down rally, July-2 closes (cron 22:52Z, applied per the F-1
circuit-breaker-fixed band — zero flags, all 22 live): TNK +5.1% and TRMD
+5.5% on the day compress both band-edge BUYs to HOLD. dNAV 0.0%, FVs
unchanged — the tape converging onto the vintage FVs (TNK to the CENT:
price $67.60 vs scenario PW FV $67.61). Both flips eyeballed + annotated
(tnk/trmd logs); 14 UNEXPLAINED all pure-price; committed SEPARATELY from
the F-13 rendering fix per the isolate-drift discipline.

Post-close actionable-long surface: SB, SBLK, ASC (+11.4%), TEN, CCEC —
TNK and TRMD age to HOLD as the market does the closing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14.25</v>
+        <v>14.86</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1481.079857180723</v>
+        <v>7407.42747318052</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.05984161039114032</v>
+        <v>0.2992899989163846</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(wo3): Phase 4 — Dorian LPG + BW LPG onboarded; v1 lock miss -> sector held PROVISIONAL
Both validators sourced in full (FY2026 10-K / Q1-2026 6-K + FY2025 20-F),
reconciled SANITY=OK (gaps -20.4%/-17.2%, k_broker ~1.2). v1 calibration lock
0/2 within ±10% -> new SECTOR_V1_UNLOCKED tier cap holds lpg at
PROVISIONAL·v1-lock-miss (guard-tested); POSITION_CYCLE_RELABEL +
OPERATING_SCRUBBER_VERIFIED extended; Cobra's filed $81.9M print replaces the
broker row; NCI-via-preferred_equity convention (BWLP $199.0M NAV-basis)
staged for owner review; 12 EV%-only price-vintage drift rows annotated
explain-not-accept. Two designed reds at HEAD await the owner ratify
(decision #1/#1b in PLAN.md).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14.86</v>
+        <v>15.32</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7407.42747318052</v>
+        <v>11814.83791587424</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.2992899989163846</v>
+        <v>0.4773671885201715</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(reweight): war-tilt regen — outputs, family re-stamps, 17 drift rows annotated; ratify staged for flip eyeball
12 material moves, all reweight/price-attributed (TEN +42% BUY headline;
every crude TRIM narrows; NAV 0.0% everywhere — weights never touch asset
NAV). Band flips vs the Friday baseline: CAPT TRIM->HOLD (reweight-driven,
in the owner-approved table) and GNK HOLD->TRIM/SHORT (price-driven, NEW —
eyeball owed). Baseline deliberately NOT ratified pending that eyeball.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -425,7 +425,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15.32</v>
+        <v>16.39</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11814.83791587424</v>
+        <v>21503.86216070459</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.4773671885201715</v>
+        <v>0.868842915584024</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(outputs): regenerate the 25-name book from clean HEAD (2343 first full surface)
book_scorecard schema 2.3, source_commit clean (WO1-F1); 2343 verdict row:
GOVERNED-WIDE·pending-anchor · HOLD · broker $0.40 (apx) · handoff-ready;
price-basis header discloses 2343 STATIC-FALLBACK until tonight's feed.
Decision-log churn is the standard per-run model-state append.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16.39</v>
+        <v>15.83</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21503.86216070459</v>
+        <v>16487.14339721867</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.868842915584024</v>
+        <v>0.666147207968431</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen at 4c658db — the book runs 2026-Q2
First committed Q2 surface: schema 2.7, balance-sheet basis 3 at Q2 + 22
lagging at Q1 (disclosed, per-row vintages), TNK VALIDATED-TIGHT (6th TIGHT),
gate 0/0. + the ASC Q2 census pins in test_scenarios (21 rows / 16 eco — the
2 NB rows carrying the once-hidden 4-hull order). Suite 632 green + 15 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-Q1</t>
+          <t>2026-Q2</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16.77122513321292</v>
+        <v>17.13246874501721</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17.81584308197886</v>
+        <v>17.37335263085518</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15.204298210064</v>
+        <v>16.77114291626024</v>
       </c>
     </row>
     <row r="9">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24201.56088373464</v>
+        <v>21596.79778295173</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.9778408437872583</v>
+        <v>0.8725978902202718</v>
       </c>
     </row>
   </sheetData>
@@ -611,7 +611,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>581.4850633114395</v>
+        <v>572.4978649978361</v>
       </c>
     </row>
     <row r="3">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>49.13333333333333</v>
+        <v>181.8600781420178</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47.214</v>
+        <v>48.138</v>
       </c>
     </row>
     <row r="5">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>119.684</v>
+        <v>125.818</v>
       </c>
     </row>
     <row r="6">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-103.359</v>
+        <v>-33.381</v>
       </c>
     </row>
     <row r="7">
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-1.746</v>
+        <v>-1.599</v>
       </c>
     </row>
     <row r="8">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0</v>
+        <v>-183.6</v>
       </c>
     </row>
     <row r="9">
@@ -712,7 +712,7 @@
         <v/>
       </c>
       <c r="B10" t="n">
-        <v>727.9113966447729</v>
+        <v>709.733943139854</v>
       </c>
     </row>
     <row r="11">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>40857533</v>
+        <v>40851870</v>
       </c>
     </row>
     <row r="12">
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>17.81584308197886</v>
+        <v>17.37335263085518</v>
       </c>
     </row>
     <row r="13">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>17.81584308197886</v>
+        <v>17.37335263085518</v>
       </c>
     </row>
     <row r="14">
@@ -772,7 +772,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
@@ -822,13 +822,13 @@
         <v>22000</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4352501465886352</v>
+        <v>0.6273651372017977</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2903118477746197</v>
+        <v>0.418452546513599</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2828355627861388</v>
+        <v>0.4076763053237459</v>
       </c>
     </row>
     <row r="3">
@@ -844,13 +844,13 @@
         <v>30000</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7843920294331035</v>
+        <v>1.046393475439435</v>
       </c>
       <c r="E3" t="n">
-        <v>0.52318948363188</v>
+        <v>0.6979444481181034</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4965894816828201</v>
+        <v>0.6624595535223631</v>
       </c>
     </row>
     <row r="4">
@@ -866,13 +866,13 @@
         <v>28000</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6971065587219865</v>
+        <v>0.9416363908800258</v>
       </c>
       <c r="E4" t="n">
-        <v>0.464970074667565</v>
+        <v>0.6280714727169773</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4299646673979741</v>
+        <v>0.5807869292706305</v>
       </c>
     </row>
     <row r="5">
@@ -888,13 +888,13 @@
         <v>19000</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3043219405219595</v>
+        <v>0.4702295103626835</v>
       </c>
       <c r="E5" t="n">
-        <v>0.202982734328147</v>
+        <v>0.3136430834119099</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1828673282235559</v>
+        <v>0.2825613364071261</v>
       </c>
     </row>
     <row r="6">
@@ -910,13 +910,13 @@
         <v>18000</v>
       </c>
       <c r="D6" t="n">
-        <v>0.260679205166401</v>
+        <v>0.4178509680829788</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1738730298459895</v>
+        <v>0.2787065957113469</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1526084209001756</v>
+        <v>0.244620879406349</v>
       </c>
     </row>
     <row r="7">
@@ -932,13 +932,13 @@
         <v>23000</v>
       </c>
       <c r="D7" t="n">
-        <v>0.4788928819441937</v>
+        <v>0.6797436794815023</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3194215522567772</v>
+        <v>0.453389034214162</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2731365048109862</v>
+        <v>0.3876917360458335</v>
       </c>
     </row>
     <row r="8">
@@ -954,13 +954,13 @@
         <v>26000</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6098210880108693</v>
+        <v>0.8368793063206164</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4067506657032499</v>
+        <v>0.5581984973158511</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3388543455548256</v>
+        <v>0.4650219469724118</v>
       </c>
     </row>
     <row r="9">
@@ -976,13 +976,13 @@
         <v>18000</v>
       </c>
       <c r="D9" t="n">
-        <v>0.260679205166401</v>
+        <v>0.4178509680829788</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1738730298459895</v>
+        <v>0.2787065957113469</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1411192515591181</v>
+        <v>0.2262045253724104</v>
       </c>
     </row>
     <row r="10">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.297975562915594</v>
+        <v>3.25702321232087</v>
       </c>
     </row>
     <row r="11">
@@ -1002,10 +1002,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>16.32221973497922</v>
+        <v>17.09088152861629</v>
       </c>
       <c r="F11" t="n">
-        <v>12.90632264714841</v>
+        <v>13.51411970393937</v>
       </c>
     </row>
     <row r="12">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>15.204298210064</v>
+        <v>16.77114291626024</v>
       </c>
     </row>
     <row r="13">
@@ -1089,19 +1089,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13.28901562086006</v>
+        <v>12.88609922381494</v>
       </c>
       <c r="C2" t="n">
-        <v>14.61567454282838</v>
+        <v>14.51188004140332</v>
       </c>
       <c r="D2" t="n">
-        <v>15.94233346479669</v>
+        <v>16.13766085899169</v>
       </c>
       <c r="E2" t="n">
-        <v>17.268992386765</v>
+        <v>17.76344167658007</v>
       </c>
       <c r="F2" t="n">
-        <v>18.59565130873331</v>
+        <v>19.38922249416843</v>
       </c>
     </row>
     <row r="3">
@@ -1111,19 +1111,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13.70346145506818</v>
+        <v>13.3835031668277</v>
       </c>
       <c r="C3" t="n">
-        <v>15.03012037703649</v>
+        <v>15.00928398441608</v>
       </c>
       <c r="D3" t="n">
-        <v>16.3567792990048</v>
+        <v>16.63506480200445</v>
       </c>
       <c r="E3" t="n">
-        <v>17.68343822097312</v>
+        <v>18.26084561959282</v>
       </c>
       <c r="F3" t="n">
-        <v>19.01009714294143</v>
+        <v>19.88662643718119</v>
       </c>
     </row>
     <row r="4">
@@ -1133,19 +1133,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14.11790728927629</v>
+        <v>13.88090710984046</v>
       </c>
       <c r="C4" t="n">
-        <v>15.44456621124461</v>
+        <v>15.50668792742884</v>
       </c>
       <c r="D4" t="n">
-        <v>16.77122513321292</v>
+        <v>17.13246874501721</v>
       </c>
       <c r="E4" t="n">
-        <v>18.09788405518123</v>
+        <v>18.75824956260558</v>
       </c>
       <c r="F4" t="n">
-        <v>19.42454297714954</v>
+        <v>20.38403038019394</v>
       </c>
     </row>
     <row r="5">
@@ -1155,19 +1155,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14.53235312348441</v>
+        <v>14.37831105285322</v>
       </c>
       <c r="C5" t="n">
-        <v>15.85901204545272</v>
+        <v>16.0040918704416</v>
       </c>
       <c r="D5" t="n">
-        <v>17.18567096742103</v>
+        <v>17.62987268802997</v>
       </c>
       <c r="E5" t="n">
-        <v>18.51232988938935</v>
+        <v>19.25565350561834</v>
       </c>
       <c r="F5" t="n">
-        <v>19.83898881135766</v>
+        <v>20.8814343232067</v>
       </c>
     </row>
     <row r="6">
@@ -1177,19 +1177,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14.94679895769252</v>
+        <v>14.87571499586598</v>
       </c>
       <c r="C6" t="n">
-        <v>16.27345787966083</v>
+        <v>16.50149581345435</v>
       </c>
       <c r="D6" t="n">
-        <v>17.60011680162914</v>
+        <v>18.12727663104273</v>
       </c>
       <c r="E6" t="n">
-        <v>18.92677572359746</v>
+        <v>19.7530574486311</v>
       </c>
       <c r="F6" t="n">
-        <v>20.25343464556577</v>
+        <v>21.37883826621946</v>
       </c>
     </row>
   </sheetData>
@@ -1227,7 +1227,7 @@
         <v>0.8</v>
       </c>
       <c r="B2" t="n">
-        <v>16.79</v>
+        <v>17.16</v>
       </c>
     </row>
     <row r="3">
@@ -1235,7 +1235,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>16.82</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="4">
@@ -1243,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>16.83</v>
+        <v>17.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean-stamp regen: Stage-A outputs (war vintage retired book-wide; BRUT/CAPT/TNK print not-actionable)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17.13246874501721</v>
+        <v>17.22201436034435</v>
       </c>
     </row>
     <row r="6">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.77114291626024</v>
+        <v>16.86889172915243</v>
       </c>
     </row>
     <row r="9">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22000</v>
+        <v>29250</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24750</v>
+        <v>29275</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.375</v>
+        <v>1.676805005952179</v>
       </c>
     </row>
     <row r="12">
@@ -552,7 +552,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>elevated</t>
+          <t>late-cycle/peak</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="14">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="15">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21596.79778295173</v>
+        <v>22102.24246494873</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8725978902202718</v>
+        <v>0.8118116395766954</v>
       </c>
     </row>
   </sheetData>
@@ -773,7 +773,7 @@
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -816,19 +816,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>22000</v>
+        <v>29300</v>
       </c>
       <c r="C2" t="n">
-        <v>22000</v>
+        <v>29300</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6273651372017977</v>
+        <v>0.8984240934992694</v>
       </c>
       <c r="E2" t="n">
-        <v>0.418452546513599</v>
+        <v>0.5992488703640128</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4076763053237459</v>
+        <v>0.583816653703862</v>
       </c>
     </row>
     <row r="3">
@@ -838,19 +838,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30000</v>
+        <v>29300</v>
       </c>
       <c r="C3" t="n">
-        <v>30000</v>
+        <v>29300</v>
       </c>
       <c r="D3" t="n">
-        <v>1.046393475439435</v>
+        <v>0.8984240934992694</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6979444481181034</v>
+        <v>0.5992488703640128</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6624595535223631</v>
+        <v>0.5687818567516555</v>
       </c>
     </row>
     <row r="4">
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28000</v>
+        <v>29250</v>
       </c>
       <c r="C4" t="n">
-        <v>28000</v>
+        <v>29250</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9416363908800258</v>
+        <v>0.8958051663852842</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6280714727169773</v>
+        <v>0.5975020459789846</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5807869292706305</v>
+        <v>0.5525189307132071</v>
       </c>
     </row>
     <row r="5">
@@ -882,19 +882,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19000</v>
+        <v>29250</v>
       </c>
       <c r="C5" t="n">
-        <v>19000</v>
+        <v>29250</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4702295103626835</v>
+        <v>0.8958051663852842</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3136430834119099</v>
+        <v>0.5975020459789846</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2825613364071261</v>
+        <v>0.5382901315125986</v>
       </c>
     </row>
     <row r="6">
@@ -904,19 +904,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18000</v>
+        <v>25000</v>
       </c>
       <c r="C6" t="n">
-        <v>18000</v>
+        <v>25000</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4178509680829788</v>
+        <v>0.689564656158947</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2787065957113469</v>
+        <v>0.4599396256580177</v>
       </c>
       <c r="F6" t="n">
-        <v>0.244620879406349</v>
+        <v>0.4036891750449185</v>
       </c>
     </row>
     <row r="7">
@@ -926,19 +926,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23000</v>
+        <v>25000</v>
       </c>
       <c r="C7" t="n">
-        <v>23000</v>
+        <v>25000</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6797436794815023</v>
+        <v>0.689564656158947</v>
       </c>
       <c r="E7" t="n">
-        <v>0.453389034214162</v>
+        <v>0.4599396256580177</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3876917360458335</v>
+        <v>0.3932931290601069</v>
       </c>
     </row>
     <row r="8">
@@ -948,19 +948,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26000</v>
+        <v>25000</v>
       </c>
       <c r="C8" t="n">
-        <v>26000</v>
+        <v>25000</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8368793063206164</v>
+        <v>0.689564656158947</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5581984973158511</v>
+        <v>0.4599396256580177</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4650219469724118</v>
+        <v>0.3831648082926146</v>
       </c>
     </row>
     <row r="9">
@@ -970,19 +970,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18000</v>
+        <v>25000</v>
       </c>
       <c r="C9" t="n">
-        <v>18000</v>
+        <v>25000</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4178509680829788</v>
+        <v>0.689564656158947</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2787065957113469</v>
+        <v>0.4599396256580177</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2262045253724104</v>
+        <v>0.37329731812192</v>
       </c>
     </row>
     <row r="10">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3.25702321232087</v>
+        <v>3.796852003200883</v>
       </c>
     </row>
     <row r="11">
@@ -1002,10 +1002,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>17.09088152861629</v>
+        <v>16.53179690486822</v>
       </c>
       <c r="F11" t="n">
-        <v>13.51411970393937</v>
+        <v>13.07203972595154</v>
       </c>
     </row>
     <row r="12">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>16.77114291626024</v>
+        <v>16.86889172915243</v>
       </c>
     </row>
     <row r="13">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>24750</v>
+        <v>29275</v>
       </c>
     </row>
   </sheetData>
@@ -1089,19 +1089,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12.88609922381494</v>
+        <v>13.08471432485743</v>
       </c>
       <c r="C2" t="n">
-        <v>14.51188004140332</v>
+        <v>14.74525114219415</v>
       </c>
       <c r="D2" t="n">
-        <v>16.13766085899169</v>
+        <v>16.40578795953086</v>
       </c>
       <c r="E2" t="n">
-        <v>17.76344167658007</v>
+        <v>18.06632477686758</v>
       </c>
       <c r="F2" t="n">
-        <v>19.38922249416843</v>
+        <v>19.72686159420428</v>
       </c>
     </row>
     <row r="3">
@@ -1111,19 +1111,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13.3835031668277</v>
+        <v>13.49282752526418</v>
       </c>
       <c r="C3" t="n">
-        <v>15.00928398441608</v>
+        <v>15.1533643426009</v>
       </c>
       <c r="D3" t="n">
-        <v>16.63506480200445</v>
+        <v>16.81390115993761</v>
       </c>
       <c r="E3" t="n">
-        <v>18.26084561959282</v>
+        <v>18.47443797727433</v>
       </c>
       <c r="F3" t="n">
-        <v>19.88662643718119</v>
+        <v>20.13497479461103</v>
       </c>
     </row>
     <row r="4">
@@ -1133,19 +1133,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13.88090710984046</v>
+        <v>13.90094072567092</v>
       </c>
       <c r="C4" t="n">
-        <v>15.50668792742884</v>
+        <v>15.56147754300764</v>
       </c>
       <c r="D4" t="n">
-        <v>17.13246874501721</v>
+        <v>17.22201436034435</v>
       </c>
       <c r="E4" t="n">
-        <v>18.75824956260558</v>
+        <v>18.88255117768107</v>
       </c>
       <c r="F4" t="n">
-        <v>20.38403038019394</v>
+        <v>20.54308799501778</v>
       </c>
     </row>
     <row r="5">
@@ -1155,19 +1155,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14.37831105285322</v>
+        <v>14.30905392607767</v>
       </c>
       <c r="C5" t="n">
-        <v>16.0040918704416</v>
+        <v>15.96959074341439</v>
       </c>
       <c r="D5" t="n">
-        <v>17.62987268802997</v>
+        <v>17.63012756075111</v>
       </c>
       <c r="E5" t="n">
-        <v>19.25565350561834</v>
+        <v>19.29066437808783</v>
       </c>
       <c r="F5" t="n">
-        <v>20.8814343232067</v>
+        <v>20.95120119542453</v>
       </c>
     </row>
     <row r="6">
@@ -1177,19 +1177,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14.87571499586598</v>
+        <v>14.71716712648442</v>
       </c>
       <c r="C6" t="n">
-        <v>16.50149581345435</v>
+        <v>16.37770394382114</v>
       </c>
       <c r="D6" t="n">
-        <v>18.12727663104273</v>
+        <v>18.03824076115785</v>
       </c>
       <c r="E6" t="n">
-        <v>19.7530574486311</v>
+        <v>19.69877757849457</v>
       </c>
       <c r="F6" t="n">
-        <v>21.37883826621946</v>
+        <v>21.35931439583128</v>
       </c>
     </row>
   </sheetData>
@@ -1227,7 +1227,7 @@
         <v>0.8</v>
       </c>
       <c r="B2" t="n">
-        <v>17.16</v>
+        <v>17.25</v>
       </c>
     </row>
     <row r="3">
@@ -1235,7 +1235,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>17.2</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="4">
@@ -1243,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>17.21</v>
+        <v>17.29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regen from clean HEAD (TRMD pair absorbed): book at the 8/28 close, 13 names Q2 vintage — surface stamp clean
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/asc_fv_report.xlsx
+++ b/outputs/asc_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17.99</v>
+        <v>17.36</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>34910.84211762037</v>
+        <v>28606.60947607103</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.28226934545007</v>
+        <v>1.050715943340518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>